<commit_message>
Fix contradictory judgment in simple validator; split into two axes
사용자 실제 입력(2.17억/10년/성과급 3,500만)에서 버퍼율 210.7%인데
"상환 능력 부족" 판정이 뜨고, 바로 아래에서는 "3.81억까지 안전"이라고
말하는 모순이 드러났다.

원인: 판정 수식이 월 수지 적자를 AND 조건으로 묶어, 누적 잉여가 아무리
커도 무조건 "부족"으로 떨어뜨렸다. 금액(얼마를 모으나)과 안정성(그 돈이
얼마나 변동적인가)은 다른 축인데 한 판정에 뭉쳐 놓은 설계 결함이다.

수정:
- 버퍼율을 둘로 분리. ① 성과급 포함, ② 성과급 0 가정
- 판정에 "금액은 충분 — 성과급 의존 주의" 단계 신설
- 연도별 표에 E·F열(성과급 0 시나리오) 추가해 ②의 근거를 노출
- 성과급 소득 비중, 한도 소진율 지표 추가
- 안전 최대 차용액을 성과급 포함/제외 두 가지로 분리
- 필요 기간에 "년차" 표기, 읽는 순서 3줄 안내 추가

한도 소진율은 무이자 한도(217,391,304원) 대비 원금 비율이다. 2.17억이면
99.8%로, 39만원만 더 빌려도 과세 구간이라 95% 초과 시 경고를 띄운다.

검증: 수식 67개 중 오류 0개. 4개 시나리오 재계산으로 판정 분기 확인.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Wn2trZJqbasDeXJ5Cs9NgB
</commit_message>
<xml_diff>
--- a/sheets/pci-loan-check/PCI_간편검증.xlsx
+++ b/sheets/pci-loan-check/PCI_간편검증.xlsx
@@ -21,7 +21,7 @@
     <numFmt numFmtId="165" formatCode="0&quot;년&quot;"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,10 +42,10 @@
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -67,8 +67,12 @@
       <b val="1"/>
       <sz val="14"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -105,6 +109,11 @@
         <fgColor rgb="00FCE4E4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E7E6E6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -132,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -140,27 +149,31 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="7" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="7" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="3" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -172,7 +185,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="7">
     <dxf>
       <font>
         <b val="1"/>
@@ -230,6 +243,14 @@
         <b val="1"/>
         <color rgb="009C0006"/>
       </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFEB9C"/>
+          <bgColor rgb="00FFEB9C"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -317,7 +338,7 @@
     </comment>
     <comment ref="B6" authorId="0" shapeId="0">
       <text>
-        <t>세후 기준입니다. 세전 금액만 안다면 대략 × 0.6 정도로 넣으세요 (과표 35% 구간 + 지방소득세 가정).</t>
+        <t>세후 기준입니다. 세전 금액만 안다면 대략 × 0.6 정도로 넣으세요.</t>
       </text>
     </comment>
     <comment ref="B12" authorId="0" shapeId="0">
@@ -325,7 +346,17 @@
         <t>0으로 두면 급여가 전혀 오르지 않는다고 보고 계산합니다. 국세청에 제시할 자료라면 0이 가장 안전합니다.</t>
       </text>
     </comment>
-    <comment ref="B26" authorId="0" shapeId="0">
+    <comment ref="B19" authorId="0" shapeId="0">
+      <text>
+        <t>성과급까지 포함한 전체 소득 기준입니다. 성과급은 이 계산에 이미 들어가 있습니다.</t>
+      </text>
+    </comment>
+    <comment ref="B25" authorId="0" shapeId="0">
+      <text>
+        <t>성과급이 한 푼도 안 나온다고 가정했을 때의 버퍼율입니다. 버퍼율 ①과 차이가 클수록 상환 계획이 성과급에 의존한다는 뜻입니다.</t>
+      </text>
+    </comment>
+    <comment ref="B32" authorId="0" shapeId="0">
       <text>
         <t>상속세 및 증여세법 시행령 제31조의4 — 적정이자율 연 4.6%. 무상대여 이익이 연 1천만원 이상이면 전액이 증여재산가액.</t>
       </text>
@@ -623,13 +654,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="46" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -778,7 +811,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>■ 결과</t>
+          <t>■ 1단계 · 금액이 되는가   (성과급 포함)</t>
         </is>
       </c>
       <c r="B14" s="3" t="n"/>
@@ -787,13 +820,18 @@
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>연간 세후 소득</t>
+          <t>연간 세후 소득 (성과급 포함)</t>
         </is>
       </c>
       <c r="B15" s="10">
         <f>$B$5*12+$B$6</f>
         <v/>
       </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>월급 12개월 + 성과급. 성과급도 당연히 포함됩니다</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
@@ -816,11 +854,6 @@
         <f>$B$15-$B$16</f>
         <v/>
       </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>음수면 애초에 상환 불가</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -829,7 +862,7 @@
         </is>
       </c>
       <c r="B18" s="11">
-        <f>INDEX($C$35:$C$44,$B$10)</f>
+        <f>INDEX($C$48:$C$57,$B$10)</f>
         <v/>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -841,7 +874,7 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>만기 상환 버퍼율</t>
+          <t>버퍼율 ①  (성과급 포함)</t>
         </is>
       </c>
       <c r="B19" s="12">
@@ -850,383 +883,609 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>100% = 딱 맞음 · 120% 이상이어야 안전</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="28" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+          <t>120% 이상이면 금액은 넉넉</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>■ 2단계 · 성과급 없이도 되는가   (안정성)</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n"/>
+      <c r="C21" s="3" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>성과급이 소득에서 차지하는 비중</t>
+        </is>
+      </c>
+      <c r="B22" s="13">
+        <f>IFERROR($B$6/$B$15,"")</f>
+        <v/>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>30% 넘으면 소명 시 약한 고리</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>월급만으로 월 수지</t>
+        </is>
+      </c>
+      <c r="B23" s="10">
+        <f>$B$5-$B$7-$B$8-ROUND($B$9*$B$11,0)/12</f>
+        <v/>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>음수면 월급으로 대출·생활비를 못 감당한다는 뜻</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>성과급 0 가정 시 누적 잉여</t>
+        </is>
+      </c>
+      <c r="B24" s="11">
+        <f>INDEX($F$48:$F$57,$B$10)</f>
+        <v/>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>성과급이 한 푼도 안 나온다고 보면</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>버퍼율 ②  (성과급 0 기준)</t>
+        </is>
+      </c>
+      <c r="B25" s="12">
+        <f>IFERROR($B$24/$B$9,"")</f>
+        <v/>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>100% 이상이면 성과급 없이도 상환 가능</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="28" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>★ 최종 판정</t>
         </is>
       </c>
-      <c r="B20" s="13">
-        <f>IF(AND($B$18&gt;=$B$9*1.2,$B$21&gt;=0),"✅ 상환 여유 충분",IF(AND($B$18&gt;=$B$9,$B$21&gt;=0),"⚠ 상환 가능 (주의 요망)","❌ 상환 능력 부족 (증여 추정 위험)"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
-        <is>
-          <t>월 수지 (성과급 빼고)</t>
-        </is>
-      </c>
-      <c r="B21" s="10">
-        <f>$B$5-$B$7-$B$8-ROUND($B$9*$B$11,0)/12</f>
-        <v/>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>성과급 없이도 흑자여야 안전</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="B27" s="14">
+        <f>IF(AND($B$19&gt;=1.2,$B$25&gt;=1),"✅ 상환 여유 충분",IF(AND($B$19&gt;=1.2,$B$25&lt;1),"⚠ 금액은 충분 — 성과급 의존 주의",IF($B$19&gt;=1,"⚠ 상환 가능 (주의 요망)","❌ 상환 능력 부족 (증여 추정 위험)")))</f>
+        <v/>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>버퍼율 ①과 ② 를 같이 보고 내린 판정</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>■ 증여세 체크</t>
         </is>
       </c>
-      <c r="B23" s="3" t="n"/>
-      <c r="C23" s="3" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="9" t="inlineStr">
+      <c r="B29" s="3" t="n"/>
+      <c r="C29" s="3" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
         <is>
           <t>무상대여 이익 (연)</t>
         </is>
       </c>
-      <c r="B24" s="14">
+      <c r="B30" s="15">
         <f>MAX(0,ROUND($B$9*0.046,0)-ROUND($B$9*$B$11,0))</f>
         <v/>
       </c>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="C30" s="6" t="inlineStr">
         <is>
           <t>법정 적정이자(4.6%) − 실제 약정이자</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="9" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
         <is>
           <t>증여세 과세 여부</t>
         </is>
       </c>
-      <c r="B25" s="15">
-        <f>IF($B$24&gt;=10000000,"❌ 과세 대상 — 이익 전액이 증여재산가액","✅ 비과세 (연 1,000만원 미만)")</f>
-        <v/>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="B31" s="16">
+        <f>IF($B$30&gt;=10000000,"❌ 과세 대상 — 이익 전액이 증여재산가액","✅ 비과세 (연 1,000만원 미만)")</f>
+        <v/>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
         <is>
           <t>1,000만원 이상이면 초과분 아닌 전액 과세</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="9" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
         <is>
           <t>무이자로 빌릴 수 있는 최대 원금</t>
         </is>
       </c>
-      <c r="B26" s="10" t="n">
+      <c r="B32" s="10" t="n">
         <v>217391304</v>
       </c>
-      <c r="C26" s="6" t="inlineStr">
+      <c r="C32" s="6" t="inlineStr">
         <is>
           <t>1,000만원 ÷ 4.6% — 고정값</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t>한도 소진율</t>
+        </is>
+      </c>
+      <c r="B33" s="17">
+        <f>IF($B$11&gt;0,"-",IFERROR($B$9/$B$32,""))</f>
+        <v/>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>100% 넘으면 증여세 과세 구간</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>■ 그래서 어떻게 하면 되나</t>
         </is>
       </c>
-      <c r="B28" s="3" t="n"/>
-      <c r="C28" s="3" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>이 조건에서 안전한 최대 차용액</t>
-        </is>
-      </c>
-      <c r="B29" s="11">
+      <c r="B35" s="3" t="n"/>
+      <c r="C35" s="3" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>안전한 최대 차용액  (성과급 포함 기준)</t>
+        </is>
+      </c>
+      <c r="B36" s="11">
         <f>ROUND($B$18/1.2,-6)</f>
         <v/>
       </c>
-      <c r="C29" s="6" t="inlineStr">
-        <is>
-          <t>백만원 단위 내림 — 여유 충분이 나오는 금액</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>성과급이 계속 나온다는 전제</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>안전한 최대 차용액  (성과급 0 기준)</t>
+        </is>
+      </c>
+      <c r="B37" s="11">
+        <f>MAX(0,ROUND($B$24/1.2,-6))</f>
+        <v/>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>성과급이 끊겨도 버티는 금액 — 진짜 보수적 안전선</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>원금을 다 갚으려면 필요한 기간</t>
         </is>
       </c>
-      <c r="B30" s="16">
-        <f>IF(COUNTIF($C$35:$C$44,"&gt;="&amp;$B$9)=0,"10년 안에는 불가",11-COUNTIF($C$35:$C$44,"&gt;="&amp;$B$9))</f>
-        <v/>
-      </c>
-      <c r="C30" s="6" t="inlineStr">
-        <is>
-          <t>누적 잉여가 원금을 넘어서는 연차</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="100" customHeight="1">
-      <c r="A31" s="9" t="inlineStr">
+      <c r="B38" s="18">
+        <f>IF(COUNTIF($C$48:$C$57,"&gt;="&amp;$B$9)=0,"10년 안에는 불가",(11-COUNTIF($C$48:$C$57,"&gt;="&amp;$B$9))&amp;"년차")</f>
+        <v/>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>성과급 포함 기준</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="118" customHeight="1">
+      <c r="A39" s="9" t="inlineStr">
         <is>
           <t>한줄 진단</t>
         </is>
       </c>
-      <c r="B31" s="17">
-        <f>IF($B$24&gt;=10000000,"⚠ 무상대여 이익 "&amp;TEXT($B$24,"#,##0")&amp;"원이 연 1,000만원 이상 → 초과분이 아닌 이익 전액이 증여재산가액으로 과세될 수 있음."&amp;CHAR(10),"")&amp;IF(AND($B$11=0,$B$9&gt;217391304),"⚠ 무이자로는 217,391,304원까지만 안전. 원금을 낮추거나 최소한의 이자를 약정하세요."&amp;CHAR(10),"")&amp;IF($B$21&lt;0,"⚠ 성과급을 빼면 월 "&amp;TEXT(ABS($B$21),"#,##0")&amp;"원 적자 → 상환 재원을 변동 성과급에 의존. 소명 시 가장 취약한 지점."&amp;CHAR(10),"")&amp;IF($B$18&lt;$B$9,"⚠ 이 조건이면 "&amp;TEXT(ROUND($B$18/1.2,-6),"#,##0")&amp;"원까지가 안전선. 원금을 줄이거나 기간을 늘리세요."&amp;CHAR(10),"")&amp;IF($B$11&gt;0,"ℹ 이자 지급 시 27.5%를 원천징수해 다음 달 10일까지 납부해야 차용으로 인정됨."&amp;CHAR(10),"")&amp;"ℹ 차용증(확정일자) + 원금 전액 계좌이체 + 매달 상환 이체기록, 이 셋이 없으면 숫자가 좋아도 소용없습니다."</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="B39" s="19">
+        <f>IF($B$30&gt;=10000000,"⚠ 무상대여 이익 "&amp;TEXT($B$30,"#,##0")&amp;"원이 연 1,000만원 이상 → 초과분이 아닌 이익 전액이 증여재산가액으로 과세될 수 있음."&amp;CHAR(10),"")&amp;IF(AND($B$11=0,$B$9&gt;$B$32),"⚠ 무이자로는 "&amp;TEXT($B$32,"#,##0")&amp;"원까지만 안전. 원금을 낮추거나 최소한의 이자를 약정하세요."&amp;CHAR(10),"")&amp;IF(AND($B$11=0,$B$9&lt;=$B$32,$B$9&gt;$B$32*0.95),"⚠ 무이자 한도를 "&amp;TEXT($B$33,"0.0%")&amp;" 소진했습니다. 원금을 "&amp;TEXT($B$32-$B$9,"#,##0")&amp;"원만 더 늘려도 증여세 과세 구간입니다."&amp;CHAR(10),"")&amp;IF(AND($B$19&gt;=1.2,$B$25&lt;1),"⚠ 성과급이 없다고 보면 버퍼율이 "&amp;TEXT($B$25,"0.0%")&amp;"로 떨어집니다. 이 계획은 성과급이 매년 나온다는 전제 위에 서 있습니다."&amp;CHAR(10),"")&amp;IF($B$23&lt;0,"⚠ 월급만으로는 월 "&amp;TEXT(ABS($B$23),"#,##0")&amp;"원 적자입니다 (대출 상환액이 실수령액에 육박하거나 넘습니다)."&amp;CHAR(10),"")&amp;IF($B$19&lt;1,"⚠ 금액 자체가 부족합니다. 이 조건이면 "&amp;TEXT(ROUND($B$18/1.2,-6),"#,##0")&amp;"원까지가 안전선입니다."&amp;CHAR(10),"")&amp;IF($B$11&gt;0,"ℹ 이자 지급 시 27.5%를 원천징수해 다음 달 10일까지 납부해야 차용으로 인정됨."&amp;CHAR(10),"")&amp;"ℹ 차용증(확정일자) + 원금 전액 계좌이체 + 매달 상환 이체기록, 이 셋이 없으면 숫자가 좋아도 소용없습니다."</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="20" t="inlineStr">
+        <is>
+          <t>■ 읽는 순서 — 이 세 줄만 보면 됩니다</t>
+        </is>
+      </c>
+      <c r="B41" s="20" t="n"/>
+      <c r="C41" s="20" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="21" t="inlineStr">
+        <is>
+          <t>1) B19 버퍼율 ① 이 120% 이상인가?   → 금액이 되는지</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="21" t="inlineStr">
+        <is>
+          <t>2) B25 버퍼율 ② 가 100% 이상인가?   → 성과급 없이도 되는지</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="21" t="inlineStr">
+        <is>
+          <t>3) B31 이 비과세인가?   → 무이자라면 원금이 B32 이하인지</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
         <is>
           <t>■ 연도별 누적  [자동 — 건드릴 것 없음]</t>
         </is>
       </c>
-      <c r="B33" s="3" t="n"/>
-      <c r="C33" s="3" t="n"/>
-      <c r="D33" s="3" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="18" t="inlineStr">
+      <c r="B46" s="3" t="n"/>
+      <c r="C46" s="3" t="n"/>
+      <c r="D46" s="3" t="n"/>
+      <c r="E46" s="3" t="n"/>
+      <c r="F46" s="3" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="22" t="inlineStr">
         <is>
           <t>연차</t>
         </is>
       </c>
-      <c r="B34" s="18" t="inlineStr">
+      <c r="B47" s="22" t="inlineStr">
         <is>
           <t>연간 잉여</t>
         </is>
       </c>
-      <c r="C34" s="18" t="inlineStr">
+      <c r="C47" s="22" t="inlineStr">
         <is>
           <t>누적 잉여</t>
         </is>
       </c>
-      <c r="D34" s="18" t="inlineStr">
+      <c r="D47" s="22" t="inlineStr">
         <is>
           <t>원금 대비</t>
         </is>
       </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="19" t="n">
+      <c r="E47" s="22" t="inlineStr">
+        <is>
+          <t>연간 잉여 (성과급 0)</t>
+        </is>
+      </c>
+      <c r="F47" s="22" t="inlineStr">
+        <is>
+          <t>누적 잉여 (성과급 0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B35" s="20">
+      <c r="B48" s="24">
         <f>ROUND($B$15*(1+$B$12)^(1-1),0)-$B$16</f>
         <v/>
       </c>
-      <c r="C35" s="20">
-        <f>B35</f>
-        <v/>
-      </c>
-      <c r="D35" s="21">
-        <f>IFERROR(C35/$B$9,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="19" t="n">
+      <c r="C48" s="24">
+        <f>B48</f>
+        <v/>
+      </c>
+      <c r="D48" s="25">
+        <f>IFERROR(C48/$B$9,"")</f>
+        <v/>
+      </c>
+      <c r="E48" s="24">
+        <f>ROUND($B$5*12*(1+$B$12)^(1-1),0)-$B$16</f>
+        <v/>
+      </c>
+      <c r="F48" s="24">
+        <f>E48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="B36" s="20">
+      <c r="B49" s="24">
         <f>ROUND($B$15*(1+$B$12)^(2-1),0)-$B$16</f>
         <v/>
       </c>
-      <c r="C36" s="20">
-        <f>C35+B36</f>
-        <v/>
-      </c>
-      <c r="D36" s="21">
-        <f>IFERROR(C36/$B$9,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="19" t="n">
+      <c r="C49" s="24">
+        <f>C48+B49</f>
+        <v/>
+      </c>
+      <c r="D49" s="25">
+        <f>IFERROR(C49/$B$9,"")</f>
+        <v/>
+      </c>
+      <c r="E49" s="24">
+        <f>ROUND($B$5*12*(1+$B$12)^(2-1),0)-$B$16</f>
+        <v/>
+      </c>
+      <c r="F49" s="24">
+        <f>F48+E49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="B37" s="20">
+      <c r="B50" s="24">
         <f>ROUND($B$15*(1+$B$12)^(3-1),0)-$B$16</f>
         <v/>
       </c>
-      <c r="C37" s="20">
-        <f>C36+B37</f>
-        <v/>
-      </c>
-      <c r="D37" s="21">
-        <f>IFERROR(C37/$B$9,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="19" t="n">
+      <c r="C50" s="24">
+        <f>C49+B50</f>
+        <v/>
+      </c>
+      <c r="D50" s="25">
+        <f>IFERROR(C50/$B$9,"")</f>
+        <v/>
+      </c>
+      <c r="E50" s="24">
+        <f>ROUND($B$5*12*(1+$B$12)^(3-1),0)-$B$16</f>
+        <v/>
+      </c>
+      <c r="F50" s="24">
+        <f>F49+E50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="B38" s="20">
+      <c r="B51" s="24">
         <f>ROUND($B$15*(1+$B$12)^(4-1),0)-$B$16</f>
         <v/>
       </c>
-      <c r="C38" s="20">
-        <f>C37+B38</f>
-        <v/>
-      </c>
-      <c r="D38" s="21">
-        <f>IFERROR(C38/$B$9,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="19" t="n">
+      <c r="C51" s="24">
+        <f>C50+B51</f>
+        <v/>
+      </c>
+      <c r="D51" s="25">
+        <f>IFERROR(C51/$B$9,"")</f>
+        <v/>
+      </c>
+      <c r="E51" s="24">
+        <f>ROUND($B$5*12*(1+$B$12)^(4-1),0)-$B$16</f>
+        <v/>
+      </c>
+      <c r="F51" s="24">
+        <f>F50+E51</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="B39" s="20">
+      <c r="B52" s="24">
         <f>ROUND($B$15*(1+$B$12)^(5-1),0)-$B$16</f>
         <v/>
       </c>
-      <c r="C39" s="20">
-        <f>C38+B39</f>
-        <v/>
-      </c>
-      <c r="D39" s="21">
-        <f>IFERROR(C39/$B$9,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="19" t="n">
+      <c r="C52" s="24">
+        <f>C51+B52</f>
+        <v/>
+      </c>
+      <c r="D52" s="25">
+        <f>IFERROR(C52/$B$9,"")</f>
+        <v/>
+      </c>
+      <c r="E52" s="24">
+        <f>ROUND($B$5*12*(1+$B$12)^(5-1),0)-$B$16</f>
+        <v/>
+      </c>
+      <c r="F52" s="24">
+        <f>F51+E52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="23" t="n">
         <v>6</v>
       </c>
-      <c r="B40" s="20">
+      <c r="B53" s="24">
         <f>ROUND($B$15*(1+$B$12)^(6-1),0)-$B$16</f>
         <v/>
       </c>
-      <c r="C40" s="20">
-        <f>C39+B40</f>
-        <v/>
-      </c>
-      <c r="D40" s="21">
-        <f>IFERROR(C40/$B$9,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="19" t="n">
+      <c r="C53" s="24">
+        <f>C52+B53</f>
+        <v/>
+      </c>
+      <c r="D53" s="25">
+        <f>IFERROR(C53/$B$9,"")</f>
+        <v/>
+      </c>
+      <c r="E53" s="24">
+        <f>ROUND($B$5*12*(1+$B$12)^(6-1),0)-$B$16</f>
+        <v/>
+      </c>
+      <c r="F53" s="24">
+        <f>F52+E53</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="23" t="n">
         <v>7</v>
       </c>
-      <c r="B41" s="20">
+      <c r="B54" s="24">
         <f>ROUND($B$15*(1+$B$12)^(7-1),0)-$B$16</f>
         <v/>
       </c>
-      <c r="C41" s="20">
-        <f>C40+B41</f>
-        <v/>
-      </c>
-      <c r="D41" s="21">
-        <f>IFERROR(C41/$B$9,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="19" t="n">
+      <c r="C54" s="24">
+        <f>C53+B54</f>
+        <v/>
+      </c>
+      <c r="D54" s="25">
+        <f>IFERROR(C54/$B$9,"")</f>
+        <v/>
+      </c>
+      <c r="E54" s="24">
+        <f>ROUND($B$5*12*(1+$B$12)^(7-1),0)-$B$16</f>
+        <v/>
+      </c>
+      <c r="F54" s="24">
+        <f>F53+E54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="23" t="n">
         <v>8</v>
       </c>
-      <c r="B42" s="20">
+      <c r="B55" s="24">
         <f>ROUND($B$15*(1+$B$12)^(8-1),0)-$B$16</f>
         <v/>
       </c>
-      <c r="C42" s="20">
-        <f>C41+B42</f>
-        <v/>
-      </c>
-      <c r="D42" s="21">
-        <f>IFERROR(C42/$B$9,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="19" t="n">
+      <c r="C55" s="24">
+        <f>C54+B55</f>
+        <v/>
+      </c>
+      <c r="D55" s="25">
+        <f>IFERROR(C55/$B$9,"")</f>
+        <v/>
+      </c>
+      <c r="E55" s="24">
+        <f>ROUND($B$5*12*(1+$B$12)^(8-1),0)-$B$16</f>
+        <v/>
+      </c>
+      <c r="F55" s="24">
+        <f>F54+E55</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="23" t="n">
         <v>9</v>
       </c>
-      <c r="B43" s="20">
+      <c r="B56" s="24">
         <f>ROUND($B$15*(1+$B$12)^(9-1),0)-$B$16</f>
         <v/>
       </c>
-      <c r="C43" s="20">
-        <f>C42+B43</f>
-        <v/>
-      </c>
-      <c r="D43" s="21">
-        <f>IFERROR(C43/$B$9,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="19" t="n">
+      <c r="C56" s="24">
+        <f>C55+B56</f>
+        <v/>
+      </c>
+      <c r="D56" s="25">
+        <f>IFERROR(C56/$B$9,"")</f>
+        <v/>
+      </c>
+      <c r="E56" s="24">
+        <f>ROUND($B$5*12*(1+$B$12)^(9-1),0)-$B$16</f>
+        <v/>
+      </c>
+      <c r="F56" s="24">
+        <f>F55+E56</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="23" t="n">
         <v>10</v>
       </c>
-      <c r="B44" s="20">
+      <c r="B57" s="24">
         <f>ROUND($B$15*(1+$B$12)^(10-1),0)-$B$16</f>
         <v/>
       </c>
-      <c r="C44" s="20">
-        <f>C43+B44</f>
-        <v/>
-      </c>
-      <c r="D44" s="21">
-        <f>IFERROR(C44/$B$9,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="6" t="inlineStr">
-        <is>
-          <t>초록색으로 칠해진 줄 = 그 해에 원금을 다 갚을 수 있다는 뜻</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="6" t="inlineStr">
+      <c r="C57" s="24">
+        <f>C56+B57</f>
+        <v/>
+      </c>
+      <c r="D57" s="25">
+        <f>IFERROR(C57/$B$9,"")</f>
+        <v/>
+      </c>
+      <c r="E57" s="24">
+        <f>ROUND($B$5*12*(1+$B$12)^(10-1),0)-$B$16</f>
+        <v/>
+      </c>
+      <c r="F57" s="24">
+        <f>F56+E57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>초록색으로 칠해진 줄 = 그 해에 원금을 다 갚을 수 있다는 뜻 (성과급 포함 기준)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>E·F열은 성과급이 한 푼도 안 나온다고 가정한 경우입니다. 이 둘의 차이가 곧 성과급 의존도입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
         <is>
           <t>연간 잉여는 소득에만 상승률을 적용하고 지출은 고정으로 둡니다 (보수적 추정).</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="22" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="26" t="inlineStr">
         <is>
           <t>※ 사전 점검용 추산입니다. 실제 과세 판단은 개별 사실관계에 좌우되므로 실행 전 세무대리인 확인을 권합니다.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="6">
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="A63:F63"/>
+    <mergeCell ref="A44:C44"/>
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="A43:C43"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
-  <conditionalFormatting sqref="B20">
+  <conditionalFormatting sqref="B27">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>ISNUMBER(SEARCH("충분",B20))</formula>
+      <formula>ISNUMBER(SEARCH("충분",B27))</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1">
-      <formula>ISNUMBER(SEARCH("주의",B20))</formula>
+      <formula>ISNUMBER(SEARCH("주의",B27))</formula>
     </cfRule>
     <cfRule type="expression" priority="3" dxfId="2">
-      <formula>ISNUMBER(SEARCH("부족",B20))</formula>
+      <formula>ISNUMBER(SEARCH("부족",B27))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B19">
@@ -1237,24 +1496,51 @@
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B25">
+    <cfRule type="cellIs" priority="6" operator="greaterThanOrEqual" dxfId="3">
+      <formula>1.2</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="7" operator="lessThan" dxfId="4">
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B17">
-    <cfRule type="cellIs" priority="6" operator="lessThan" dxfId="5">
+    <cfRule type="cellIs" priority="8" operator="lessThan" dxfId="5">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B21">
-    <cfRule type="cellIs" priority="7" operator="lessThan" dxfId="5">
+  <conditionalFormatting sqref="B23">
+    <cfRule type="cellIs" priority="9" operator="lessThan" dxfId="5">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B25">
-    <cfRule type="expression" priority="8" dxfId="2">
-      <formula>ISNUMBER(SEARCH("과세 대상",B25))</formula>
+  <conditionalFormatting sqref="E48:F57">
+    <cfRule type="cellIs" priority="10" operator="lessThan" dxfId="5">
+      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A35:D44">
-    <cfRule type="expression" priority="9" dxfId="3">
-      <formula>$C35&gt;=$B$9</formula>
+  <conditionalFormatting sqref="B22">
+    <cfRule type="cellIs" priority="11" operator="greaterThanOrEqual" dxfId="6">
+      <formula>0.3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B31">
+    <cfRule type="expression" priority="12" dxfId="2">
+      <formula>ISNUMBER(SEARCH("과세 대상",B31))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B33">
+    <cfRule type="cellIs" priority="13" operator="greaterThan" dxfId="4">
+      <formula>1</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="14" operator="between" dxfId="6">
+      <formula>0.95</formula>
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A48:F57">
+    <cfRule type="expression" priority="15" dxfId="3">
+      <formula>$C48&gt;=$B$9</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">

</xml_diff>